<commit_message>
Guests: invite type, plus-ones from placeholder rows, and RSVP reset
- Invite type per guest (ceremony or reception), seeded from the old
  Ceremony flag. Filter by it, switch one guest by clicking their tag,
  or set every guest in the selected households at once.
- The spreadsheet's "Guest" / "Guest <host>" rows become a plus-one
  allowance on their host with no name, so the guest types it in when
  they RSVP. A migration converts rows already in the database; the
  importer does the same on re-import.
- Reset RSVP (per household, or in bulk) puts guests and plus-ones back
  to awaiting reply and clears what the RSVP form filled in, for testing
  and for un-RSVPing someone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xs2LEQN3LS8KLzmeNc5hhk
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_wedding.xlsx
+++ b/tests/fixtures/sample_wedding.xlsx
@@ -870,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1189,69 +1189,108 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>H-002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Guest</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Guest Jordan Sample</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Bride</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>H-003</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Riley</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>O'Placeholder</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Bride</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
         <v>1</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Riley O'Placeholder</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Riley</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>3 Demo Rd</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Ogdenville</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="S6" t="n">
         <v>46203</v>
       </c>
     </row>

</xml_diff>